<commit_message>
Add silicon economy layer while preserving 13+3 plan
Append 13-direction silicon mapping, five agent-economy opportunities, eight evaluation metrics, and synchronized PDF, Excel, and XMind.
</commit_message>
<xml_diff>
--- a/AI投资决策与财务模型.xlsx
+++ b/AI投资决策与财务模型.xlsx
@@ -2,17 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb30446313d96429c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R00b49e0abcc54539"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating_Model" sheetId="3" r:id="Re381a305cdd14981"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment_Map" sheetId="4" r:id="Rf8557b4634cf4af8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capital_Themes" sheetId="5" r:id="R718d55004a614289"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence_Maturity" sheetId="6" r:id="Rb751ff40a7cd4f5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorecard" sheetId="7" r:id="R355c9324e3864d8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stress_Test" sheetId="8" r:id="R8e9dcf57f85248e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Due_Diligence" sheetId="9" r:id="Rd0d02c6bbe4b4893"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R16d9f41a76384f37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="11" r:id="R3b90a81da97542d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8857851cfb954800"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rb7eaa636d05a46a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating_Model" sheetId="3" r:id="Rf9b23b8f1bf345d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment_Map" sheetId="4" r:id="R49b7c417156e45c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capital_Themes" sheetId="5" r:id="R33f1a70c0a1e4880"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence_Maturity" sheetId="6" r:id="R2959a3347a484745"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorecard" sheetId="7" r:id="R1f8a93186f1a49ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stress_Test" sheetId="8" r:id="R5eab07cfcf5c4234"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Silicon_Economy" sheetId="9" r:id="R5874c98190984111"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Due_Diligence" sheetId="10" r:id="R5414c355faa845a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="11" r:id="R5bf557a035f141e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="12" r:id="R5a7ed465da914cce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -869,6 +870,349 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>项目与公司尽调清单</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="4"/>
+      <x:c r="B2" s="4"/>
+      <x:c r="C2" s="4"/>
+      <x:c r="D2" s="4"/>
+      <x:c r="E2" s="4"/>
+      <x:c r="F2" s="4"/>
+      <x:c r="G2" s="4"/>
+      <x:c r="H2" s="4"/>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A4" s="13" t="str">
+        <x:v>模块</x:v>
+      </x:c>
+      <x:c r="B4" s="14" t="str">
+        <x:v>检查事项</x:v>
+      </x:c>
+      <x:c r="C4" s="14" t="str">
+        <x:v>证据</x:v>
+      </x:c>
+      <x:c r="D4" s="14" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+      <x:c r="E4" s="14" t="str">
+        <x:v>优先级</x:v>
+      </x:c>
+      <x:c r="F4" s="14" t="str">
+        <x:v>负责人</x:v>
+      </x:c>
+      <x:c r="G4" s="14" t="str">
+        <x:v>截止日</x:v>
+      </x:c>
+      <x:c r="H4" s="15" t="str">
+        <x:v>结论/风险</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A5" s="23" t="str">
+        <x:v>客户</x:v>
+      </x:c>
+      <x:c r="B5" s="23" t="str">
+        <x:v>前三大客户、合同、发票、回款流水</x:v>
+      </x:c>
+      <x:c r="C5" s="23" t="str">
+        <x:v>合同+银行流水</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="G5" s="73"/>
+      <x:c r="H5" s="23" t="str"/>
+    </x:row>
+    <x:row r="6" ht="66" hidden="0" customHeight="1">
+      <x:c r="A6" s="24" t="str">
+        <x:v>产品</x:v>
+      </x:c>
+      <x:c r="B6" s="24" t="str">
+        <x:v>真实使用频次、留存、失败率、部署周期</x:v>
+      </x:c>
+      <x:c r="C6" s="24" t="str">
+        <x:v>后台数据+客户访谈</x:v>
+      </x:c>
+      <x:c r="D6" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="E6" s="24" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="F6" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="G6" s="74"/>
+      <x:c r="H6" s="24" t="str"/>
+    </x:row>
+    <x:row r="7" ht="66" hidden="0" customHeight="1">
+      <x:c r="A7" s="24" t="str">
+        <x:v>财务</x:v>
+      </x:c>
+      <x:c r="B7" s="24" t="str">
+        <x:v>收入确认、毛利、现金消耗、应收账龄</x:v>
+      </x:c>
+      <x:c r="C7" s="24" t="str">
+        <x:v>总账+审计底稿</x:v>
+      </x:c>
+      <x:c r="D7" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="E7" s="24" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="F7" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="G7" s="74"/>
+      <x:c r="H7" s="24" t="str"/>
+    </x:row>
+    <x:row r="8" ht="66" hidden="0" customHeight="1">
+      <x:c r="A8" s="24" t="str">
+        <x:v>技术</x:v>
+      </x:c>
+      <x:c r="B8" s="24" t="str">
+        <x:v>模型依赖、推理成本、代码质量、容灾</x:v>
+      </x:c>
+      <x:c r="C8" s="24" t="str">
+        <x:v>架构图+代码审计</x:v>
+      </x:c>
+      <x:c r="D8" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="E8" s="24" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="F8" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="G8" s="74"/>
+      <x:c r="H8" s="24" t="str"/>
+    </x:row>
+    <x:row r="9" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A9" s="24" t="str">
+        <x:v>数据</x:v>
+      </x:c>
+      <x:c r="B9" s="24" t="str">
+        <x:v>授权、来源、跨境、个人信息处理</x:v>
+      </x:c>
+      <x:c r="C9" s="24" t="str">
+        <x:v>数据清单+授权协议</x:v>
+      </x:c>
+      <x:c r="D9" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="E9" s="24" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="F9" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="G9" s="74"/>
+      <x:c r="H9" s="24" t="str"/>
+    </x:row>
+    <x:row r="10" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A10" s="24" t="str">
+        <x:v>知识产权</x:v>
+      </x:c>
+      <x:c r="B10" s="24" t="str">
+        <x:v>代码、商标、专利、开源许可证</x:v>
+      </x:c>
+      <x:c r="C10" s="24" t="str">
+        <x:v>权属文件+SBOM</x:v>
+      </x:c>
+      <x:c r="D10" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="E10" s="24" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="F10" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="G10" s="74"/>
+      <x:c r="H10" s="24" t="str"/>
+    </x:row>
+    <x:row r="11" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A11" s="24" t="str">
+        <x:v>合规</x:v>
+      </x:c>
+      <x:c r="B11" s="24" t="str">
+        <x:v>备案、牌照、内容安全、行业监管</x:v>
+      </x:c>
+      <x:c r="C11" s="24" t="str">
+        <x:v>官方文件+法律意见</x:v>
+      </x:c>
+      <x:c r="D11" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="E11" s="24" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="F11" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="G11" s="74"/>
+      <x:c r="H11" s="24" t="str"/>
+    </x:row>
+    <x:row r="12" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A12" s="24" t="str">
+        <x:v>团队</x:v>
+      </x:c>
+      <x:c r="B12" s="24" t="str">
+        <x:v>履历、诚信、关键人、招聘与激励</x:v>
+      </x:c>
+      <x:c r="C12" s="24" t="str">
+        <x:v>背调+访谈</x:v>
+      </x:c>
+      <x:c r="D12" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="E12" s="24" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="F12" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="G12" s="74"/>
+      <x:c r="H12" s="24" t="str"/>
+    </x:row>
+    <x:row r="13" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A13" s="24" t="str">
+        <x:v>股权</x:v>
+      </x:c>
+      <x:c r="B13" s="24" t="str">
+        <x:v>股东名册、期权池、历史融资、代持</x:v>
+      </x:c>
+      <x:c r="C13" s="24" t="str">
+        <x:v>工商+股权文件</x:v>
+      </x:c>
+      <x:c r="D13" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="E13" s="24" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="F13" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="G13" s="74"/>
+      <x:c r="H13" s="24" t="str"/>
+    </x:row>
+    <x:row r="14" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A14" s="24" t="str">
+        <x:v>条款</x:v>
+      </x:c>
+      <x:c r="B14" s="24" t="str">
+        <x:v>清算优先、反稀释、回购、信息权</x:v>
+      </x:c>
+      <x:c r="C14" s="24" t="str">
+        <x:v>TS+章程</x:v>
+      </x:c>
+      <x:c r="D14" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="E14" s="24" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="F14" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="G14" s="74"/>
+      <x:c r="H14" s="24" t="str"/>
+    </x:row>
+    <x:row r="15" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A15" s="24" t="str">
+        <x:v>竞争</x:v>
+      </x:c>
+      <x:c r="B15" s="24" t="str">
+        <x:v>国内外竞品、大厂进入、开源替代</x:v>
+      </x:c>
+      <x:c r="C15" s="24" t="str">
+        <x:v>竞品矩阵+客户访谈</x:v>
+      </x:c>
+      <x:c r="D15" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="E15" s="24" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="F15" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="G15" s="74"/>
+      <x:c r="H15" s="24" t="str"/>
+    </x:row>
+    <x:row r="16" ht="66" hidden="0" customHeight="1">
+      <x:c r="A16" s="25" t="str">
+        <x:v>退出</x:v>
+      </x:c>
+      <x:c r="B16" s="25" t="str">
+        <x:v>下一轮融资、并购方、上市与转让限制</x:v>
+      </x:c>
+      <x:c r="C16" s="25" t="str">
+        <x:v>资本规划+条款</x:v>
+      </x:c>
+      <x:c r="D16" s="25" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="E16" s="25" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="F16" s="25" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="G16" s="75"/>
+      <x:c r="H16" s="25" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+  </x:mergeCells>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="D5:D16">
+      <x:formula1>"待开始,进行中,已完成,阻塞"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E5:E16">
+      <x:formula1>"高,中,低"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="50" hidden="0" customWidth="1"/>
@@ -1202,7 +1546,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -4427,19 +4771,19 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>项目与公司尽调清单</x:v>
+        <x:v>硅基经济层｜AI作为经济参与者</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -4460,308 +4804,267 @@
       <x:c r="H2" s="4"/>
     </x:row>
     <x:row r="3"/>
-    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="13" t="str">
-        <x:v>模块</x:v>
+        <x:v>新增方向</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
-        <x:v>检查事项</x:v>
+        <x:v>产品核心</x:v>
       </x:c>
       <x:c r="C4" s="14" t="str">
-        <x:v>证据</x:v>
+        <x:v>首要客户</x:v>
       </x:c>
       <x:c r="D4" s="14" t="str">
+        <x:v>商业模式</x:v>
+      </x:c>
+      <x:c r="E4" s="14" t="str">
+        <x:v>90天证据</x:v>
+      </x:c>
+      <x:c r="F4" s="14" t="str">
+        <x:v>关键指标</x:v>
+      </x:c>
+      <x:c r="G4" s="14" t="str">
+        <x:v>人类控制</x:v>
+      </x:c>
+      <x:c r="H4" s="15" t="str">
         <x:v>状态</x:v>
-      </x:c>
-      <x:c r="E4" s="14" t="str">
-        <x:v>优先级</x:v>
-      </x:c>
-      <x:c r="F4" s="14" t="str">
-        <x:v>负责人</x:v>
-      </x:c>
-      <x:c r="G4" s="14" t="str">
-        <x:v>截止日</x:v>
-      </x:c>
-      <x:c r="H4" s="15" t="str">
-        <x:v>结论/风险</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A5" s="23" t="str">
-        <x:v>客户</x:v>
+        <x:v>AI智能体身份与授权网络</x:v>
       </x:c>
       <x:c r="B5" s="23" t="str">
-        <x:v>前三大客户、合同、发票、回款流水</x:v>
+        <x:v>身份、代表关系、权限、撤销与审计</x:v>
       </x:c>
       <x:c r="C5" s="23" t="str">
-        <x:v>合同+银行流水</x:v>
+        <x:v>平台、金融、企业软件</x:v>
       </x:c>
       <x:c r="D5" s="23" t="str">
-        <x:v>待开始</x:v>
+        <x:v>调用计费＋企业订阅</x:v>
       </x:c>
       <x:c r="E5" s="23" t="str">
-        <x:v>高</x:v>
+        <x:v>一个真实平台授权与撤销闭环</x:v>
       </x:c>
       <x:c r="F5" s="23" t="str">
-        <x:v>待定</x:v>
-      </x:c>
-      <x:c r="G5" s="73"/>
-      <x:c r="H5" s="23" t="str"/>
-    </x:row>
-    <x:row r="6" ht="66" hidden="0" customHeight="1">
+        <x:v>身份覆盖率、撤销时延</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="str">
+        <x:v>绑定合法人/组织，可随时撤销</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="str">
+        <x:v>研究</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A6" s="24" t="str">
-        <x:v>产品</x:v>
+        <x:v>AI长期记忆与数字人格托管</x:v>
       </x:c>
       <x:c r="B6" s="24" t="str">
-        <x:v>真实使用频次、留存、失败率、部署周期</x:v>
+        <x:v>跨模型保存、迁移、继承和删除记忆</x:v>
       </x:c>
       <x:c r="C6" s="24" t="str">
-        <x:v>后台数据+客户访谈</x:v>
+        <x:v>个人AI、企业Agent、教育养老</x:v>
       </x:c>
       <x:c r="D6" s="24" t="str">
-        <x:v>待开始</x:v>
+        <x:v>存储订阅＋迁移＋治理</x:v>
       </x:c>
       <x:c r="E6" s="24" t="str">
-        <x:v>高</x:v>
+        <x:v>跨两种模型迁移并可控删除</x:v>
       </x:c>
       <x:c r="F6" s="24" t="str">
-        <x:v>待定</x:v>
-      </x:c>
-      <x:c r="G6" s="74"/>
-      <x:c r="H6" s="24" t="str"/>
-    </x:row>
-    <x:row r="7" ht="66" hidden="0" customHeight="1">
+        <x:v>记忆命中率、迁移成功率</x:v>
+      </x:c>
+      <x:c r="G6" s="24" t="str">
+        <x:v>所有者可导出、删除和停止</x:v>
+      </x:c>
+      <x:c r="H6" s="24" t="str">
+        <x:v>研究</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A7" s="24" t="str">
-        <x:v>财务</x:v>
+        <x:v>Agent-to-Agent交易与结算</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
-        <x:v>收入确认、毛利、现金消耗、应收账龄</x:v>
+        <x:v>机器采购、托管、验收、付款与争议</x:v>
       </x:c>
       <x:c r="C7" s="24" t="str">
-        <x:v>总账+审计底稿</x:v>
+        <x:v>API平台、跨境服务、机器人运营商</x:v>
       </x:c>
       <x:c r="D7" s="24" t="str">
-        <x:v>待开始</x:v>
+        <x:v>交易费＋托管费＋风控</x:v>
       </x:c>
       <x:c r="E7" s="24" t="str">
-        <x:v>高</x:v>
+        <x:v>两个智能体可追责小额交易</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
-        <x:v>待定</x:v>
-      </x:c>
-      <x:c r="G7" s="74"/>
-      <x:c r="H7" s="24" t="str"/>
-    </x:row>
-    <x:row r="8" ht="66" hidden="0" customHeight="1">
+        <x:v>成功率、退款率、争议率</x:v>
+      </x:c>
+      <x:c r="G7" s="24" t="str">
+        <x:v>预算上限、人工批准和追责</x:v>
+      </x:c>
+      <x:c r="H7" s="24" t="str">
+        <x:v>研究</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A8" s="24" t="str">
-        <x:v>技术</x:v>
+        <x:v>AI信誉、责任与任务保险</x:v>
       </x:c>
       <x:c r="B8" s="24" t="str">
-        <x:v>模型依赖、推理成本、代码质量、容灾</x:v>
+        <x:v>历史表现、风险评分和失败保障</x:v>
       </x:c>
       <x:c r="C8" s="24" t="str">
-        <x:v>架构图+代码审计</x:v>
+        <x:v>企业采购、平台、保险</x:v>
       </x:c>
       <x:c r="D8" s="24" t="str">
-        <x:v>待开始</x:v>
+        <x:v>评分API＋保费分成</x:v>
       </x:c>
       <x:c r="E8" s="24" t="str">
-        <x:v>高</x:v>
+        <x:v>评分模型和保险/平台合作意向</x:v>
       </x:c>
       <x:c r="F8" s="24" t="str">
-        <x:v>待定</x:v>
-      </x:c>
-      <x:c r="G8" s="74"/>
-      <x:c r="H8" s="24" t="str"/>
-    </x:row>
-    <x:row r="9" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A9" s="24" t="str">
-        <x:v>数据</x:v>
-      </x:c>
-      <x:c r="B9" s="24" t="str">
-        <x:v>授权、来源、跨境、个人信息处理</x:v>
-      </x:c>
-      <x:c r="C9" s="24" t="str">
-        <x:v>数据清单+授权协议</x:v>
-      </x:c>
-      <x:c r="D9" s="24" t="str">
-        <x:v>待开始</x:v>
-      </x:c>
-      <x:c r="E9" s="24" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="F9" s="24" t="str">
-        <x:v>待定</x:v>
-      </x:c>
-      <x:c r="G9" s="74"/>
-      <x:c r="H9" s="24" t="str"/>
-    </x:row>
-    <x:row r="10" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A10" s="24" t="str">
-        <x:v>知识产权</x:v>
-      </x:c>
-      <x:c r="B10" s="24" t="str">
-        <x:v>代码、商标、专利、开源许可证</x:v>
-      </x:c>
-      <x:c r="C10" s="24" t="str">
-        <x:v>权属文件+SBOM</x:v>
-      </x:c>
-      <x:c r="D10" s="24" t="str">
-        <x:v>待开始</x:v>
-      </x:c>
-      <x:c r="E10" s="24" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="F10" s="24" t="str">
-        <x:v>待定</x:v>
-      </x:c>
-      <x:c r="G10" s="74"/>
-      <x:c r="H10" s="24" t="str"/>
-    </x:row>
-    <x:row r="11" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A11" s="24" t="str">
-        <x:v>合规</x:v>
-      </x:c>
-      <x:c r="B11" s="24" t="str">
-        <x:v>备案、牌照、内容安全、行业监管</x:v>
-      </x:c>
-      <x:c r="C11" s="24" t="str">
-        <x:v>官方文件+法律意见</x:v>
-      </x:c>
-      <x:c r="D11" s="24" t="str">
-        <x:v>待开始</x:v>
-      </x:c>
-      <x:c r="E11" s="24" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="F11" s="24" t="str">
-        <x:v>待定</x:v>
-      </x:c>
-      <x:c r="G11" s="74"/>
-      <x:c r="H11" s="24" t="str"/>
-    </x:row>
-    <x:row r="12" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A12" s="24" t="str">
-        <x:v>团队</x:v>
-      </x:c>
-      <x:c r="B12" s="24" t="str">
-        <x:v>履历、诚信、关键人、招聘与激励</x:v>
-      </x:c>
-      <x:c r="C12" s="24" t="str">
-        <x:v>背调+访谈</x:v>
-      </x:c>
-      <x:c r="D12" s="24" t="str">
-        <x:v>待开始</x:v>
-      </x:c>
-      <x:c r="E12" s="24" t="str">
-        <x:v>中</x:v>
-      </x:c>
-      <x:c r="F12" s="24" t="str">
-        <x:v>待定</x:v>
-      </x:c>
-      <x:c r="G12" s="74"/>
-      <x:c r="H12" s="24" t="str"/>
-    </x:row>
-    <x:row r="13" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A13" s="24" t="str">
-        <x:v>股权</x:v>
-      </x:c>
-      <x:c r="B13" s="24" t="str">
-        <x:v>股东名册、期权池、历史融资、代持</x:v>
-      </x:c>
-      <x:c r="C13" s="24" t="str">
-        <x:v>工商+股权文件</x:v>
-      </x:c>
-      <x:c r="D13" s="24" t="str">
-        <x:v>待开始</x:v>
-      </x:c>
-      <x:c r="E13" s="24" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="F13" s="24" t="str">
-        <x:v>待定</x:v>
-      </x:c>
-      <x:c r="G13" s="74"/>
-      <x:c r="H13" s="24" t="str"/>
-    </x:row>
-    <x:row r="14" ht="52.79999923706055" hidden="0" customHeight="1">
+        <x:v>任务成功率、赔付率</x:v>
+      </x:c>
+      <x:c r="G8" s="24" t="str">
+        <x:v>高风险任务强制人工批准</x:v>
+      </x:c>
+      <x:c r="H8" s="24" t="str">
+        <x:v>研究</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="66" hidden="0" customHeight="1">
+      <x:c r="A9" s="25" t="str">
+        <x:v>AI能力市场与工具供应链</x:v>
+      </x:c>
+      <x:c r="B9" s="25" t="str">
+        <x:v>发现、测试、采购和替换模型/API/工具</x:v>
+      </x:c>
+      <x:c r="C9" s="25" t="str">
+        <x:v>开发者、Agent平台、企业IT</x:v>
+      </x:c>
+      <x:c r="D9" s="25" t="str">
+        <x:v>佣金＋治理＋认证</x:v>
+      </x:c>
+      <x:c r="E9" s="25" t="str">
+        <x:v>20个工具接入和恶意工具拦截</x:v>
+      </x:c>
+      <x:c r="F9" s="25" t="str">
+        <x:v>替换成功率、供应商集中度</x:v>
+      </x:c>
+      <x:c r="G9" s="25" t="str">
+        <x:v>最小权限、白名单和调用审计</x:v>
+      </x:c>
+      <x:c r="H9" s="25" t="str">
+        <x:v>研究</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10"/>
+    <x:row r="11"/>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="13" t="str">
+        <x:v>硅基评估指标</x:v>
+      </x:c>
+      <x:c r="B12" s="14" t="str">
+        <x:v>核心问题</x:v>
+      </x:c>
+      <x:c r="C12" s="15" t="str">
+        <x:v>量化指标</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A13" s="23" t="str">
+        <x:v>自主程度</x:v>
+      </x:c>
+      <x:c r="B13" s="23" t="str">
+        <x:v>无人干预能完成多少任务</x:v>
+      </x:c>
+      <x:c r="C13" s="23" t="str">
+        <x:v>任务闭环率、人工接管率</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A14" s="24" t="str">
-        <x:v>条款</x:v>
+        <x:v>持续身份</x:v>
       </x:c>
       <x:c r="B14" s="24" t="str">
-        <x:v>清算优先、反稀释、回购、信息权</x:v>
+        <x:v>是否有稳定身份与历史</x:v>
       </x:c>
       <x:c r="C14" s="24" t="str">
-        <x:v>TS+章程</x:v>
-      </x:c>
-      <x:c r="D14" s="24" t="str">
-        <x:v>待开始</x:v>
-      </x:c>
-      <x:c r="E14" s="24" t="str">
-        <x:v>高</x:v>
-      </x:c>
-      <x:c r="F14" s="24" t="str">
-        <x:v>待定</x:v>
-      </x:c>
-      <x:c r="G14" s="74"/>
-      <x:c r="H14" s="24" t="str"/>
-    </x:row>
-    <x:row r="15" ht="52.79999923706055" hidden="0" customHeight="1">
+        <x:v>身份覆盖率、撤销时间</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A15" s="24" t="str">
-        <x:v>竞争</x:v>
+        <x:v>长期记忆</x:v>
       </x:c>
       <x:c r="B15" s="24" t="str">
-        <x:v>国内外竞品、大厂进入、开源替代</x:v>
+        <x:v>状态能否跨模型延续</x:v>
       </x:c>
       <x:c r="C15" s="24" t="str">
-        <x:v>竞品矩阵+客户访谈</x:v>
-      </x:c>
-      <x:c r="D15" s="24" t="str">
-        <x:v>待开始</x:v>
-      </x:c>
-      <x:c r="E15" s="24" t="str">
-        <x:v>中</x:v>
-      </x:c>
-      <x:c r="F15" s="24" t="str">
-        <x:v>待定</x:v>
-      </x:c>
-      <x:c r="G15" s="74"/>
-      <x:c r="H15" s="24" t="str"/>
-    </x:row>
-    <x:row r="16" ht="66" hidden="0" customHeight="1">
-      <x:c r="A16" s="25" t="str">
-        <x:v>退出</x:v>
-      </x:c>
-      <x:c r="B16" s="25" t="str">
-        <x:v>下一轮融资、并购方、上市与转让限制</x:v>
-      </x:c>
-      <x:c r="C16" s="25" t="str">
-        <x:v>资本规划+条款</x:v>
-      </x:c>
-      <x:c r="D16" s="25" t="str">
-        <x:v>待开始</x:v>
-      </x:c>
-      <x:c r="E16" s="25" t="str">
-        <x:v>中</x:v>
-      </x:c>
-      <x:c r="F16" s="25" t="str">
-        <x:v>待定</x:v>
-      </x:c>
-      <x:c r="G16" s="75"/>
-      <x:c r="H16" s="25" t="str"/>
+        <x:v>命中率、迁移成功率</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A16" s="24" t="str">
+        <x:v>机器支付</x:v>
+      </x:c>
+      <x:c r="B16" s="24" t="str">
+        <x:v>能否在授权预算内采购</x:v>
+      </x:c>
+      <x:c r="C16" s="24" t="str">
+        <x:v>支付成功率、争议率</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A17" s="24" t="str">
+        <x:v>多智能体协作</x:v>
+      </x:c>
+      <x:c r="B17" s="24" t="str">
+        <x:v>能否委派、验收和追责</x:v>
+      </x:c>
+      <x:c r="C17" s="24" t="str">
+        <x:v>验收率、责任链完整率</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A18" s="24" t="str">
+        <x:v>可迁移性</x:v>
+      </x:c>
+      <x:c r="B18" s="24" t="str">
+        <x:v>能否更换模型、云和工具</x:v>
+      </x:c>
+      <x:c r="C18" s="24" t="str">
+        <x:v>迁移时间、集中度</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A19" s="24" t="str">
+        <x:v>人类控制</x:v>
+      </x:c>
+      <x:c r="B19" s="24" t="str">
+        <x:v>能否暂停、撤销和接管</x:v>
+      </x:c>
+      <x:c r="C19" s="24" t="str">
+        <x:v>阻断延迟、越权事件</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A20" s="25" t="str">
+        <x:v>硅基单位经济</x:v>
+      </x:c>
+      <x:c r="B20" s="25" t="str">
+        <x:v>有效任务消耗多少资源</x:v>
+      </x:c>
+      <x:c r="C20" s="25" t="str">
+        <x:v>每任务Token、电力、资金和毛利</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
-  <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="D5:D16">
-      <x:formula1>"待开始,进行中,已完成,阻塞"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="E5:E16">
-      <x:formula1>"高,中,低"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add investor, project factory, and solo-company layers
Preserve the complete 13+3 and silicon-economy content while adding investor positioning, project generation, virtual project cards, solo-company execution, synchronized PDF, Excel, and XMind.
</commit_message>
<xml_diff>
--- a/AI投资决策与财务模型.xlsx
+++ b/AI投资决策与财务模型.xlsx
@@ -2,18 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8857851cfb954800"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rb7eaa636d05a46a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating_Model" sheetId="3" r:id="Rf9b23b8f1bf345d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment_Map" sheetId="4" r:id="R49b7c417156e45c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capital_Themes" sheetId="5" r:id="R33f1a70c0a1e4880"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence_Maturity" sheetId="6" r:id="R2959a3347a484745"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorecard" sheetId="7" r:id="R1f8a93186f1a49ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stress_Test" sheetId="8" r:id="R5eab07cfcf5c4234"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Silicon_Economy" sheetId="9" r:id="R5874c98190984111"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Due_Diligence" sheetId="10" r:id="R5414c355faa845a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="11" r:id="R5bf557a035f141e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="12" r:id="R5a7ed465da914cce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R814a183c7f0b4e09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rbb7e0701f41842e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating_Model" sheetId="3" r:id="R7444226c7f2f4ea7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment_Map" sheetId="4" r:id="R30b1124a83234cf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capital_Themes" sheetId="5" r:id="R36d81e4ce2894a2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence_Maturity" sheetId="6" r:id="Rc88017e675ba400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorecard" sheetId="7" r:id="R077afff1a2b5481d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stress_Test" sheetId="8" r:id="R5f094f3bf35f496c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Silicon_Economy" sheetId="9" r:id="Refbeeff1db70467e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Factory" sheetId="10" r:id="Rf029ef46115b4124"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solo_Company" sheetId="11" r:id="R8cd83b96b32b4b61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Due_Diligence" sheetId="12" r:id="R25b0b6c439044072"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="13" r:id="Ra2f4f3435c1342c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="14" r:id="Raf5b2b577151498a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -164,7 +166,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="81">
+  <x:cellXfs count="83">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -362,6 +364,12 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="205" fontId="3" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -869,6 +877,728 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="32" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>项目工厂｜从方向到可投资项目</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+      <x:c r="I1" s="4"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="4"/>
+      <x:c r="B2" s="4"/>
+      <x:c r="C2" s="4"/>
+      <x:c r="D2" s="4"/>
+      <x:c r="E2" s="4"/>
+      <x:c r="F2" s="4"/>
+      <x:c r="G2" s="4"/>
+      <x:c r="H2" s="4"/>
+      <x:c r="I2" s="4"/>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="13" t="str">
+        <x:v>阶段</x:v>
+      </x:c>
+      <x:c r="B4" s="14" t="str">
+        <x:v>时间</x:v>
+      </x:c>
+      <x:c r="C4" s="14" t="str">
+        <x:v>核心动作</x:v>
+      </x:c>
+      <x:c r="D4" s="14" t="str">
+        <x:v>必须产出</x:v>
+      </x:c>
+      <x:c r="E4" s="14" t="str">
+        <x:v>继续条件</x:v>
+      </x:c>
+      <x:c r="F4" s="14" t="str">
+        <x:v>停止条件</x:v>
+      </x:c>
+      <x:c r="G4" s="14" t="str">
+        <x:v>负责人</x:v>
+      </x:c>
+      <x:c r="H4" s="14" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+      <x:c r="I4" s="15" t="str">
+        <x:v>证据链接</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A5" s="23" t="str">
+        <x:v>方向验证</x:v>
+      </x:c>
+      <x:c r="B5" s="23" t="str">
+        <x:v>第1—15天</x:v>
+      </x:c>
+      <x:c r="C5" s="23" t="str">
+        <x:v>锁定客户和高频问题</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="str">
+        <x:v>客户名单、访谈提纲、10次访谈</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="str">
+        <x:v>问题高频且存在预算</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="str">
+        <x:v>问题低频或无预算</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="I5" s="23" t="str"/>
+    </x:row>
+    <x:row r="6" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A6" s="24" t="str">
+        <x:v>需求验证</x:v>
+      </x:c>
+      <x:c r="B6" s="24" t="str">
+        <x:v>第16—30天</x:v>
+      </x:c>
+      <x:c r="C6" s="24" t="str">
+        <x:v>核验痛点、预算和采购流程</x:v>
+      </x:c>
+      <x:c r="D6" s="24" t="str">
+        <x:v>30次访谈、3个明确需求</x:v>
+      </x:c>
+      <x:c r="E6" s="24" t="str">
+        <x:v>客户愿意试用或共创</x:v>
+      </x:c>
+      <x:c r="F6" s="24" t="str">
+        <x:v>30次访谈无付费需求</x:v>
+      </x:c>
+      <x:c r="G6" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="H6" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="I6" s="24" t="str"/>
+    </x:row>
+    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A7" s="24" t="str">
+        <x:v>团队招募</x:v>
+      </x:c>
+      <x:c r="B7" s="24" t="str">
+        <x:v>第1—45天</x:v>
+      </x:c>
+      <x:c r="C7" s="24" t="str">
+        <x:v>筛选创始人并试合作</x:v>
+      </x:c>
+      <x:c r="D7" s="24" t="str">
+        <x:v>候选清单、能力验证、分工</x:v>
+      </x:c>
+      <x:c r="E7" s="24" t="str">
+        <x:v>技术与行业能力可覆盖</x:v>
+      </x:c>
+      <x:c r="F7" s="24" t="str">
+        <x:v>无人愿意全职负责</x:v>
+      </x:c>
+      <x:c r="G7" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="H7" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="I7" s="24" t="str"/>
+    </x:row>
+    <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A8" s="24" t="str">
+        <x:v>原型开发</x:v>
+      </x:c>
+      <x:c r="B8" s="24" t="str">
+        <x:v>第31—60天</x:v>
+      </x:c>
+      <x:c r="C8" s="24" t="str">
+        <x:v>完成单一闭环MVP</x:v>
+      </x:c>
+      <x:c r="D8" s="24" t="str">
+        <x:v>可演示原型、测试记录</x:v>
+      </x:c>
+      <x:c r="E8" s="24" t="str">
+        <x:v>客户愿意真实试用</x:v>
+      </x:c>
+      <x:c r="F8" s="24" t="str">
+        <x:v>60天无可用产品</x:v>
+      </x:c>
+      <x:c r="G8" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="H8" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="I8" s="24" t="str"/>
+    </x:row>
+    <x:row r="9" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A9" s="24" t="str">
+        <x:v>商业验证</x:v>
+      </x:c>
+      <x:c r="B9" s="24" t="str">
+        <x:v>第61—90天</x:v>
+      </x:c>
+      <x:c r="C9" s="24" t="str">
+        <x:v>定价、试点和回款</x:v>
+      </x:c>
+      <x:c r="D9" s="24" t="str">
+        <x:v>合同/发票/回款或采购意向</x:v>
+      </x:c>
+      <x:c r="E9" s="24" t="str">
+        <x:v>至少1个付费证据</x:v>
+      </x:c>
+      <x:c r="F9" s="24" t="str">
+        <x:v>90天无付款或强意向</x:v>
+      </x:c>
+      <x:c r="G9" s="24" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="H9" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="I9" s="24" t="str"/>
+    </x:row>
+    <x:row r="10" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A10" s="25" t="str">
+        <x:v>投资准备</x:v>
+      </x:c>
+      <x:c r="B10" s="25" t="str">
+        <x:v>第90天后</x:v>
+      </x:c>
+      <x:c r="C10" s="25" t="str">
+        <x:v>公司、股权、预算、TS、数据室</x:v>
+      </x:c>
+      <x:c r="D10" s="25" t="str">
+        <x:v>完整项目档案</x:v>
+      </x:c>
+      <x:c r="E10" s="25" t="str">
+        <x:v>通过正式尽调</x:v>
+      </x:c>
+      <x:c r="F10" s="25" t="str">
+        <x:v>权属、诚信或经济性不成立</x:v>
+      </x:c>
+      <x:c r="G10" s="25" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="H10" s="25" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="I10" s="25" t="str"/>
+    </x:row>
+    <x:row r="11"/>
+    <x:row r="12"/>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="13" t="str">
+        <x:v>年度漏斗</x:v>
+      </x:c>
+      <x:c r="B13" s="14" t="str">
+        <x:v>接触人数</x:v>
+      </x:c>
+      <x:c r="C13" s="14" t="str">
+        <x:v>有效访谈</x:v>
+      </x:c>
+      <x:c r="D13" s="14" t="str">
+        <x:v>方向假设</x:v>
+      </x:c>
+      <x:c r="E13" s="14" t="str">
+        <x:v>原型</x:v>
+      </x:c>
+      <x:c r="F13" s="14" t="str">
+        <x:v>付费试点</x:v>
+      </x:c>
+      <x:c r="G13" s="15" t="str">
+        <x:v>孵化公司</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A14" s="80" t="str">
+        <x:v>计划值（非已实现）</x:v>
+      </x:c>
+      <x:c r="B14" s="80" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C14" s="80" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="D14" s="80" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E14" s="80" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F14" s="80" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G14" s="80" t="str">
+        <x:v>1—2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15"/>
+    <x:row r="16"/>
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A17" s="37" t="str">
+        <x:v>项目来源：大模型/云生态、上市公司创新需求、高校科研、连续创业者、企业未解决需求、海外成熟产品中国化或出海。</x:v>
+      </x:c>
+      <x:c r="B17" s="37"/>
+      <x:c r="C17" s="37"/>
+      <x:c r="D17" s="37"/>
+      <x:c r="E17" s="37"/>
+      <x:c r="F17" s="37"/>
+      <x:c r="G17" s="37"/>
+      <x:c r="H17" s="37"/>
+      <x:c r="I17" s="37"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:I2"/>
+    <x:mergeCell ref="A17:I17"/>
+  </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="H5:H10">
+      <x:formula1>"待开始,进行中,通过,停止"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>一人公司机会地图｜创始人 + AI 智能体</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="4"/>
+      <x:c r="B2" s="4"/>
+      <x:c r="C2" s="4"/>
+      <x:c r="D2" s="4"/>
+      <x:c r="E2" s="4"/>
+      <x:c r="F2" s="4"/>
+      <x:c r="G2" s="4"/>
+      <x:c r="H2" s="4"/>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="13" t="str">
+        <x:v>等级</x:v>
+      </x:c>
+      <x:c r="B4" s="14" t="str">
+        <x:v>方向</x:v>
+      </x:c>
+      <x:c r="C4" s="14" t="str">
+        <x:v>最小切口</x:v>
+      </x:c>
+      <x:c r="D4" s="14" t="str">
+        <x:v>首版周期</x:v>
+      </x:c>
+      <x:c r="E4" s="14" t="str">
+        <x:v>首道预算</x:v>
+      </x:c>
+      <x:c r="F4" s="14" t="str">
+        <x:v>90天证据</x:v>
+      </x:c>
+      <x:c r="G4" s="14" t="str">
+        <x:v>主要风险</x:v>
+      </x:c>
+      <x:c r="H4" s="15" t="str">
+        <x:v>结论</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A5" s="23" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="B5" s="23" t="str">
+        <x:v>API自动维护</x:v>
+      </x:c>
+      <x:c r="C5" s="23" t="str">
+        <x:v>单一API生态</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="str">
+        <x:v>2—4周</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="str">
+        <x:v>1—3万元</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="str">
+        <x:v>20个仓库、3个深度试用、1个回款</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="str">
+        <x:v>误修和代码权限</x:v>
+      </x:c>
+      <x:c r="H5" s="23" t="str">
+        <x:v>最优先</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A6" s="24" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="B6" s="24" t="str">
+        <x:v>小软件专属云</x:v>
+      </x:c>
+      <x:c r="C6" s="24" t="str">
+        <x:v>现有云上的部署管理层</x:v>
+      </x:c>
+      <x:c r="D6" s="24" t="str">
+        <x:v>3—6周</x:v>
+      </x:c>
+      <x:c r="E6" s="24" t="str">
+        <x:v>3—10万元</x:v>
+      </x:c>
+      <x:c r="F6" s="24" t="str">
+        <x:v>20个活跃项目、5个付费客户</x:v>
+      </x:c>
+      <x:c r="G6" s="24" t="str">
+        <x:v>支持成本和安全责任</x:v>
+      </x:c>
+      <x:c r="H6" s="24" t="str">
+        <x:v>优先</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A7" s="24" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="B7" s="24" t="str">
+        <x:v>AI能力市场</x:v>
+      </x:c>
+      <x:c r="C7" s="24" t="str">
+        <x:v>工具监测、测试和替代推荐</x:v>
+      </x:c>
+      <x:c r="D7" s="24" t="str">
+        <x:v>2—4周</x:v>
+      </x:c>
+      <x:c r="E7" s="24" t="str">
+        <x:v>1—3万元</x:v>
+      </x:c>
+      <x:c r="F7" s="24" t="str">
+        <x:v>20个工具接入、首个订阅客户</x:v>
+      </x:c>
+      <x:c r="G7" s="24" t="str">
+        <x:v>双边市场冷启动</x:v>
+      </x:c>
+      <x:c r="H7" s="24" t="str">
+        <x:v>先目录后市场</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A8" s="24" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="B8" s="24" t="str">
+        <x:v>AI私人老师</x:v>
+      </x:c>
+      <x:c r="C8" s="24" t="str">
+        <x:v>单一人群与单一结果</x:v>
+      </x:c>
+      <x:c r="D8" s="24" t="str">
+        <x:v>3—6周</x:v>
+      </x:c>
+      <x:c r="E8" s="24" t="str">
+        <x:v>1—5万元</x:v>
+      </x:c>
+      <x:c r="F8" s="24" t="str">
+        <x:v>30个家庭试用、10个付费</x:v>
+      </x:c>
+      <x:c r="G8" s="24" t="str">
+        <x:v>获客和效果证明</x:v>
+      </x:c>
+      <x:c r="H8" s="24" t="str">
+        <x:v>可验证</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A9" s="24" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="B9" s="24" t="str">
+        <x:v>AI原生合规</x:v>
+      </x:c>
+      <x:c r="C9" s="24" t="str">
+        <x:v>单一法规或垂直行业</x:v>
+      </x:c>
+      <x:c r="D9" s="24" t="str">
+        <x:v>4—8周</x:v>
+      </x:c>
+      <x:c r="E9" s="24" t="str">
+        <x:v>3—10万元</x:v>
+      </x:c>
+      <x:c r="F9" s="24" t="str">
+        <x:v>30条规则、1个回款客户</x:v>
+      </x:c>
+      <x:c r="G9" s="24" t="str">
+        <x:v>专业责任和人工交付</x:v>
+      </x:c>
+      <x:c r="H9" s="24" t="str">
+        <x:v>专业复核</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A10" s="24" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="B10" s="24" t="str">
+        <x:v>AI长期记忆</x:v>
+      </x:c>
+      <x:c r="C10" s="24" t="str">
+        <x:v>导出、整理、迁移和删除</x:v>
+      </x:c>
+      <x:c r="D10" s="24" t="str">
+        <x:v>3—6周</x:v>
+      </x:c>
+      <x:c r="E10" s="24" t="str">
+        <x:v>1—5万元</x:v>
+      </x:c>
+      <x:c r="F10" s="24" t="str">
+        <x:v>跨模型迁移、首个付费用户</x:v>
+      </x:c>
+      <x:c r="G10" s="24" t="str">
+        <x:v>隐私与安全</x:v>
+      </x:c>
+      <x:c r="H10" s="24" t="str">
+        <x:v>可验证</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A11" s="24" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="B11" s="24" t="str">
+        <x:v>身份/数据/银发/消费</x:v>
+      </x:c>
+      <x:c r="C11" s="24" t="str">
+        <x:v>SDK、管理软件或轻服务</x:v>
+      </x:c>
+      <x:c r="D11" s="24" t="str">
+        <x:v>6—12周</x:v>
+      </x:c>
+      <x:c r="E11" s="24" t="str">
+        <x:v>5—15万元</x:v>
+      </x:c>
+      <x:c r="F11" s="24" t="str">
+        <x:v>一个窄场景付费闭环</x:v>
+      </x:c>
+      <x:c r="G11" s="24" t="str">
+        <x:v>线下责任与集成</x:v>
+      </x:c>
+      <x:c r="H11" s="24" t="str">
+        <x:v>限软件层</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A12" s="25" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="B12" s="25" t="str">
+        <x:v>国防硬件/海上数据中心</x:v>
+      </x:c>
+      <x:c r="C12" s="25" t="str">
+        <x:v>研究或产业合作</x:v>
+      </x:c>
+      <x:c r="D12" s="25" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="E12" s="25" t="str">
+        <x:v>不建议单人投入</x:v>
+      </x:c>
+      <x:c r="F12" s="25" t="str">
+        <x:v>合规合作方与订单路径</x:v>
+      </x:c>
+      <x:c r="G12" s="25" t="str">
+        <x:v>重资产、资质、审批</x:v>
+      </x:c>
+      <x:c r="H12" s="25" t="str">
+        <x:v>不直接进入</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13"/>
+    <x:row r="14"/>
+    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A15" s="13" t="str">
+        <x:v>预算闸门</x:v>
+      </x:c>
+      <x:c r="B15" s="14" t="str">
+        <x:v>累计预算上限</x:v>
+      </x:c>
+      <x:c r="C15" s="14" t="str">
+        <x:v>放行证据</x:v>
+      </x:c>
+      <x:c r="D15" s="15" t="str">
+        <x:v>未达标动作</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A16" s="23" t="str">
+        <x:v>闸门1</x:v>
+      </x:c>
+      <x:c r="B16" s="23" t="str">
+        <x:v>1—3万元</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="str">
+        <x:v>明确需求和可演示原型</x:v>
+      </x:c>
+      <x:c r="D16" s="23" t="str">
+        <x:v>停止或换切口</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A17" s="24" t="str">
+        <x:v>闸门2</x:v>
+      </x:c>
+      <x:c r="B17" s="24" t="str">
+        <x:v>10万元</x:v>
+      </x:c>
+      <x:c r="C17" s="24" t="str">
+        <x:v>真实试用和安全文档需求</x:v>
+      </x:c>
+      <x:c r="D17" s="24" t="str">
+        <x:v>暂停产品化投入</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A18" s="25" t="str">
+        <x:v>闸门3</x:v>
+      </x:c>
+      <x:c r="B18" s="25" t="str">
+        <x:v>30万元</x:v>
+      </x:c>
+      <x:c r="C18" s="25" t="str">
+        <x:v>回款、续费和正贡献毛利</x:v>
+      </x:c>
+      <x:c r="D18" s="25" t="str">
+        <x:v>不扩大规模</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19"/>
+    <x:row r="20"/>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="13" t="str">
+        <x:v>时间</x:v>
+      </x:c>
+      <x:c r="B21" s="14" t="str">
+        <x:v>动作</x:v>
+      </x:c>
+      <x:c r="C21" s="14" t="str">
+        <x:v>目标</x:v>
+      </x:c>
+      <x:c r="D21" s="15" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A22" s="23" t="str">
+        <x:v>1—15天</x:v>
+      </x:c>
+      <x:c r="B22" s="23" t="str">
+        <x:v>访谈和问题库</x:v>
+      </x:c>
+      <x:c r="C22" s="23" t="str">
+        <x:v>20名访谈、50个问题</x:v>
+      </x:c>
+      <x:c r="D22" s="23" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A23" s="24" t="str">
+        <x:v>16—30天</x:v>
+      </x:c>
+      <x:c r="B23" s="24" t="str">
+        <x:v>完成MVP</x:v>
+      </x:c>
+      <x:c r="C23" s="24" t="str">
+        <x:v>核心闭环可演示</x:v>
+      </x:c>
+      <x:c r="D23" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A24" s="24" t="str">
+        <x:v>31—60天</x:v>
+      </x:c>
+      <x:c r="B24" s="24" t="str">
+        <x:v>邀请试用</x:v>
+      </x:c>
+      <x:c r="C24" s="24" t="str">
+        <x:v>10个试用、3个深度使用</x:v>
+      </x:c>
+      <x:c r="D24" s="24" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A25" s="25" t="str">
+        <x:v>61—90天</x:v>
+      </x:c>
+      <x:c r="B25" s="25" t="str">
+        <x:v>计费、安全、案例、续费</x:v>
+      </x:c>
+      <x:c r="C25" s="25" t="str">
+        <x:v>至少1个付费客户</x:v>
+      </x:c>
+      <x:c r="D25" s="25" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+  </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="D22:D25">
+      <x:formula1>"待开始,进行中,通过,停止"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
@@ -1208,7 +1938,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1546,7 +2276,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1736,18 +2466,18 @@
     <x:row r="10"/>
     <x:row r="11"/>
     <x:row r="12" ht="16.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A12" s="80" t="str">
+      <x:c r="A12" s="82" t="str">
         <x:v>MODEL STATUS</x:v>
       </x:c>
-      <x:c r="B12" s="80"/>
-      <x:c r="C12" s="80"/>
-      <x:c r="D12" s="80"/>
-      <x:c r="E12" s="80"/>
-      <x:c r="F12" s="80" t="str">
+      <x:c r="B12" s="82"/>
+      <x:c r="C12" s="82"/>
+      <x:c r="D12" s="82"/>
+      <x:c r="E12" s="82"/>
+      <x:c r="F12" s="82" t="str">
         <x:f>IF(COUNTIF(F5:F9,"FAIL")=0,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="G12" s="80"/>
+      <x:c r="G12" s="82"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>